<commit_message>
feat(lib): add translations for cyfun-small-self-assessment
</commit_message>
<xml_diff>
--- a/tools/excel/ccb/cyfun-small-self-assessment_new.xlsx
+++ b/tools/excel/ccb/cyfun-small-self-assessment_new.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="library_meta" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="requirements_meta" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="requirements_content" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="scores_meta" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="scores_content" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="library_meta" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="requirements_meta" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="requirements_content" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="scores_meta" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="scores_content" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -448,7 +448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:B17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -481,10 +481,8 @@
           <t>version</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="B3" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="4">
@@ -582,6 +580,84 @@
       <c r="B11" t="inlineStr">
         <is>
           <t>intuitem</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>name[fr]</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>CCB CyberFondamentaux Small - Auto-évaluation</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>name[nl]</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>CCB CyberFundamentals Small - Zelfbeoordeling</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>name[de]</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>CCB Cyber-Grundlagen Small - Selbstbewertung</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>description[fr]</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Centre pour la Cybersécurité Belgique - Cadre des CyberFondamentaux - Small
+Avec le contenu du site safeOnWeb en date de juillet 2025
+https://ccb.belgium.be</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>description[nl]</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Centrum voor Cyberveiligheid België - CyberFundamentals Framework - Small
+Met inhoud van de safeOnWeb website per juli 2025
+https://ccb.belgium.be</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>description[de]</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Zentrum für Cybersicherheit Belgien - Cyber-Grundlagen Framework - Small
+Mit Inhalten der safeOnWeb Website ab Juli 2025
+https://ccb.belgium.be</t>
         </is>
       </c>
     </row>
@@ -596,7 +672,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -704,6 +780,78 @@
       <c r="B9" t="inlineStr">
         <is>
           <t>scores</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>name[fr]</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>CCB CyberFondamentaux Small - Auto-évaluation</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>name[nl]</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>CCB CyberFundamentals Small - Zelfbeoordeling</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>name[de]</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>CCB Cyber-Grundlagen Small - Selbstbewertung</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>description[fr]</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Centre pour la Cybersécurité Belgique - Cadre des CyberFondamentaux - Small</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>description[nl]</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Centrum voor Cyberveiligheid België - CyberFundamentals Framework - Small</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>description[de]</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Zentrum für Cybersicherheit Belgien - Cyber-Grundlagen Framework - Small</t>
         </is>
       </c>
     </row>
@@ -718,7 +866,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:N9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -745,6 +893,51 @@
       <c r="E1" t="inlineStr">
         <is>
           <t>annotation</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>name[fr]</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>name[nl]</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>name[de]</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>description[fr]</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>description[nl]</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>description[de]</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>annotation[fr]</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>annotation[nl]</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>annotation[de]</t>
         </is>
       </c>
     </row>
@@ -776,6 +969,63 @@
 5: Two-factor authentication is in place for all critical systems.</t>
         </is>
       </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>MOTS DE PASSE</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>WACHTWOORDEN</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>PASSWÖRTER</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Avez-vous des règles en place pour vos mots de passe ?</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Heeft u regels voor uw wachtwoorden?</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Haben Sie Regeln für Ihre Passwörter?</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>1 : Pas de règles, les mots de passe n'ont aucun critère de création ou de réutilisation.
+2 : Il existe quelques règles concernant la création de mots de passe, mais pas de vérification de l'historique ou de la réutilisation.
+3 : Il existe des exigences communes pour tous les mots de passe et ceux-ci doivent être modifiés régulièrement.
+4 : Il existe des exigences strictes pour tous les utilisateurs et la plupart des systèmes, et les mots de passe ne sont modifiés qu'en cas d'indication de violation.
+5 : L'authentification multifactorielle est en place pour tous les systèmes critiques.</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>1: Geen regels, wachtwoorden hebben geen criteria voor aanmaak of hergebruik.
+2: Er zijn enkele regels rond het aanmaken van wachtwoorden, maar geen controle op geschiedenis of hergebruik.
+3: Er zijn gemeenschappelijke vereisten voor alle wachtwoorden en deze moeten regelmatig worden gewijzigd.
+4: Er zijn strenge vereisten voor alle gebruikers en de meeste systemen, en wachtwoorden worden alleen gewijzigd bij een indicatie van een schending.
+5: Multifactorauthenticatie is ingesteld voor alle kritieke systemen.</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>1: Keine Regeln, Passwörter haben keine Erstellungs- oder Wiederverwendungskriterien.
+2: Es gibt einige Regeln zur Passworterstellung, aber keine Überprüfung des Verlaufs oder der Wiederverwendung.
+3: Es gibt gemeinsame Anforderungen für alle Passwörter und diese sollten regelmäßig geändert werden.
+4: Es gibt strenge Anforderungen für alle Benutzer und die meisten Systeme, und Passwörter werden nur bei Anzeichen einer Verletzung geändert.
+5: Multi-Faktor-Authentifizierung ist für alle kritischen Systeme eingerichtet.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -805,6 +1055,63 @@
 5: All updates are done continuously and systematically, and are tested before implementation.</t>
         </is>
       </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>MAINTENANCE DES SYSTÈMES</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>SYSTEEMONDERHOUD</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>SYSTEMWARTUNG</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Mettez-vous à jour vos systèmes et applications ?</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Werkt u uw systemen en applicaties bij?</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Aktualisieren Sie Ihre Systeme und Anwendungen?</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>1 : Non, nous ne faisons aucune mise à jour tant que les systèmes continuent de fonctionner.
+2 : Des mises à jour manuelles sont effectuées en cas de besoin ou pour les systèmes les plus critiques.
+3 : Il existe une procédure standard pour la planification des mises à jour.
+4 : Tous les systèmes sont rapidement mis à jour vers leurs dernières versions.
+5 : Toutes les mises à jour sont effectuées de manière continue et systématique, et sont testées avant la mise en œuvre.</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>1: Nee, we doen geen updates zolang de systemen blijven werken.
+2: Handmatige updates worden gedaan wanneer dat nodig is of voor de meest kritieke systemen.
+3: Er is een standaardprocedure voor het plannen van updates.
+4: Alle systemen worden snel bijgewerkt naar de nieuwste versies.
+5: Alle updates worden continu en systematisch uitgevoerd en worden getest voor implementatie.</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>1: Nein, wir führen keine Updates durch, solange die Systeme weiter funktionieren.
+2: Manuelle Updates werden bei Bedarf oder für die kritischsten Systeme durchgeführt.
+3: Es gibt ein Standardverfahren für die Planung von Updates.
+4: Alle Systeme werden schnell auf die neuesten Versionen aktualisiert.
+5: Alle Updates werden kontinuierlich und systematisch durchgeführt und vor der Implementierung getestet.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -834,6 +1141,63 @@
 5: On all systems and updated daily. Suspicious activity is also reported.</t>
         </is>
       </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>GESTION ANTIVIRUS ET ANTI-MALWARE</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>ANTIVIRUS- EN ANTI-MALWAREBEHEER</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>ANTIVIRUS- UND ANTI-MALWARE-VERWALTUNG</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Disposez-vous d'un logiciel antivirus ou anti-malware ?</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Heeft u antivirus- of anti-malwaresoftware geïnstalleerd?</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Haben Sie Antivirus- oder Anti-Malware-Software installiert?</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>1 : Non, aucun.
+2 : Sur certains systèmes principaux, mais pas partout.
+3 : Sur tous les systèmes, mais ils ne sont pas nécessairement mis à jour.
+4 : Sur tous les systèmes et mis à jour plusieurs fois par semaine.
+5 : Sur tous les systèmes et mis à jour quotidiennement. Les activités suspectes sont également signalées.</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>1: Nee, geen.
+2: Op sommige belangrijke systemen, maar niet overal.
+3: Op alle systemen, maar ze worden niet noodzakelijk bijgewerkt.
+4: Op alle systemen en meerdere keren per week bijgewerkt.
+5: Op alle systemen en dagelijks bijgewerkt. Verdachte activiteiten worden ook gemeld.</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>1: Nein, keine.
+2: Auf einigen wichtigen Systemen, aber nicht überall.
+3: Auf allen Systemen, aber sie werden nicht unbedingt aktualisiert.
+4: Auf allen Systemen und mehrmals pro Woche aktualisiert.
+5: Auf allen Systemen und täglich aktualisiert. Verdächtige Aktivitäten werden ebenfalls gemeldet.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -863,6 +1227,63 @@
 5: The network is compartmentalized into strictly separated areas; anomalies are quickly detected and resolved.</t>
         </is>
       </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>SÉCURITÉ DU RÉSEAU</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>NETWERKBEVEILIGING</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>NETZWERKSICHERHEIT</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Protégez-vous votre réseau ?</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Beveiligt u uw netwerk?</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Schützen Sie Ihr Netzwerk?</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>1 : Pas activement : le réseau n'est pas segmenté et est connecté à internet sans mises à jour ni mots de passe forts.
+2 : De manière limitée : les réseaux public et interne sont séparés et protégés par un pare-feu.
+3 : Protection de base : un certain nombre de segmentations existent selon les fonctions et les besoins, et tout est documenté.
+4 : La sécurité du réseau est mesurée et surveillée ; les anomalies peuvent être détectées.
+5 : Le réseau est compartimenté en zones strictement séparées ; les anomalies sont rapidement détectées et résolues.</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>1: Niet actief: het netwerk is niet gesegmenteerd en is verbonden met het internet zonder updates en sterke wachtwoorden.
+2: Op een beperkte manier: het publieke en interne netwerk zijn gescheiden en beschermd door een firewall.
+3: Basisbescherming: er bestaan een aantal segmentaties volgens functies en behoeften en alles is gedocumenteerd.
+4: De beveiliging van het netwerk wordt gemeten en bewaakt; afwijkingen kunnen worden gedetecteerd.
+5: Het netwerk is opgedeeld in strikt gescheiden zones; afwijkingen worden snel gedetecteerd en opgelost.</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>1: Nicht aktiv: Das Netzwerk ist nicht segmentiert und ohne Updates und starke Passwörter mit dem Internet verbunden.
+2: In begrenztem Maße: Das öffentliche und das interne Netzwerk sind getrennt und durch eine Firewall geschützt.
+3: Grundschutz: Es gibt eine Reihe von Segmentierungen nach Funktionen und Bedürfnissen, und alles ist dokumentiert.
+4: Die Sicherheit des Netzwerks wird gemessen und überwacht; Anomalien können erkannt werden.
+5: Das Netzwerk ist in streng getrennte Bereiche unterteilt; Anomalien werden schnell erkannt und behoben.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -892,6 +1313,63 @@
 5: All data is backed up completely with fast recovery time and without data loss.</t>
         </is>
       </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>PROCÉDURE DE SAUVEGARDE</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>BACK-UPPROCEDURE</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>BACKUP-VERFAHREN</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Disposez-vous d'une procédure de sauvegarde ?</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Heeft u een back-upprocedure?</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>Haben Sie ein Backup-Verfahren?</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>1 : Non, ni systématique ni documentée.
+2 : Les sauvegardes sont limitées et manuelles, et la restauration n'est pas testée. Parfois, les sauvegardes sont faites localement par les employés eux-mêmes, sur des clés USB ou des disques durs externes.
+3 : Les sauvegardes sont testées et disponibles pour tous les systèmes principaux, et les restaurations de fichiers sont testées régulièrement.
+4 : Les sauvegardes sont chiffrées, disponibles pour tous les systèmes de l'organisation et testées immédiatement avec des indicateurs de performance à améliorer.
+5 : Toutes les données sont sauvegardées complètement avec un temps de récupération rapide et sans perte de données.</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>1: Nee, niet systematisch noch gedocumenteerd.
+2: Back-ups zijn beperkt en handmatig, en herstel wordt niet getest. Soms worden de back-ups lokaal door de medewerkers zelf gemaakt, op USB-sticks of externe harde schijven.
+3: Back-ups worden getest en zijn beschikbaar voor alle belangrijke systemen, en bestandsherstel wordt regelmatig getest.
+4: Back-ups zijn versleuteld, beschikbaar voor alle systemen in de organisatie en onmiddellijk getest met prestatie-indicatoren om te verbeteren.
+5: Alle gegevens worden volledig geback-upt met snelle hersteltijd en zonder gegevensverlies.</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>1: Nein, weder systematisch noch dokumentiert.
+2: Backups sind begrenzt und manuell, und die Wiederherstellung wird nicht getestet. Manchmal werden die Backups von den Mitarbeitern selbst lokal auf USB-Sticks oder externen Festplatten erstellt.
+3: Backups werden getestet und sind für alle wichtigen Systeme verfügbar, und Dateiwiederherstellungen werden regelmäßig getestet.
+4: Backups sind verschlüsselt, für alle Systeme in der Organisation verfügbar und werden sofort getestet, mit Leistungskennzahlen zur Verbesserung.
+5: Alle Daten werden vollständig gesichert mit schneller Wiederherstellungszeit und ohne Datenverlust.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -921,6 +1399,63 @@
 5: Administrator accounts are disabled or modified if there are changes and anomalies.</t>
         </is>
       </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>DROITS D'ADMINISTRATION</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>ADMINISTRATIERECHTEN</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>VERWALTUNGSRECHTE</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Comment protégez-vous vos comptes administrateur ?</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>Hoe beschermt u uw beheerdersaccounts?</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>Wie schützen Sie Ihre Administratorkonten?</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>1 : Sans vue d'ensemble de nos comptes administrateurs ; nous ne les protégeons pas spécifiquement.
+2 : Nous gérons l'accès administrateur uniquement sur certains services.
+3 : Tous les accès administrateur sont distribués dans des comptes séparés et gérés de manière centralisée.
+4 : Tous les comptes administrateur sont strictement surveillés avec des notifications automatiques en cas d'anomalies.
+5 : Les comptes administrateur sont désactivés ou modifiés en cas de changements et d'anomalies.</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>1: Zonder overzicht van onze beheerdersaccounts; we beschermen ze niet specifiek.
+2: We beheren beheerderstoegang alleen op bepaalde diensten.
+3: Alle beheerderstoegang is verdeeld over afzonderlijke accounts en wordt centraal beheerd.
+4: Alle beheerdersaccounts worden strikt bewaakt met automatische meldingen bij afwijkingen.
+5: Beheerdersaccounts worden uitgeschakeld of gewijzigd bij veranderingen en afwijkingen.</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>1: Ohne Überblick über unsere Administratorkonten; wir schützen sie nicht speziell.
+2: Wir verwalten den Administratorzugang nur bei bestimmten Diensten.
+3: Alle Administratorzugänge sind auf separate Konten verteilt und werden zentral verwaltet.
+4: Alle Administratorkonten werden streng überwacht, mit automatischen Benachrichtigungen bei Anomalien.
+5: Administratorkonten werden bei Änderungen und Anomalien deaktiviert oder geändert.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -950,6 +1485,63 @@
 5: Access control is centralized, regularly reviewed and follows the life cycle of employees (entry/change of position/exit).</t>
         </is>
       </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>SÉCURITÉ PHYSIQUE</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>FYSIEKE BEVEILIGING</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>PHYSISCHE SICHERHEIT</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Avez-vous des mesures en place pour protéger physiquement l'accès à vos locaux et à votre infrastructure ?</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Heeft u maatregelen getroffen om de fysieke toegang tot uw gebouwen en infrastructuur te beschermen?</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>Haben Sie Maßnahmen getroffen, um den physischen Zugang zu Ihren Räumlichkeiten und Ihrer Infrastruktur zu schützen?</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>1 : Nous n'avons rien en place.
+2 : Nous ne protégeons que les systèmes critiques (par ex. la salle des serveurs).
+3 : Toute notre infrastructure est protégée, y compris la protection contre les incendies et les inondations.
+4 : Nous contrôlons l'accès de manière centralisée (par ex. badges) et segmentons l'accès selon les niveaux de confidentialité.
+5 : Le contrôle d'accès est centralisé, régulièrement revu et suit le cycle de vie des employés (entrée/changement de poste/sortie).</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>1: We hebben niets in plaats.
+2: We beschermen alleen kritieke systemen (bijv. serverruimte).
+3: Al onze infrastructuur is beschermd, inclusief brand- en overstromingsbescherming.
+4: We controleren de toegang centraal (bijv. badges) en segmenteren de toegang op basis van vertrouwelijkheidsniveaus.
+5: Toegangscontrole is gecentraliseerd, wordt regelmatig herzien en volgt de levenscyclus van medewerkers (in dienst/functiewijziging/uit dienst).</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>1: Wir haben nichts eingerichtet.
+2: Wir schützen nur kritische Systeme (z.B. Serverraum).
+3: Unsere gesamte Infrastruktur ist geschützt, einschließlich Brand- und Hochwasserschutz.
+4: Wir kontrollieren den Zugang zentral (z.B. Badges) und segmentieren den Zugang nach Vertraulichkeitsstufen.
+5: Die Zugangskontrolle ist zentralisiert, wird regelmäßig überprüft und folgt dem Lebenszyklus der Mitarbeiter (Eintritt/Positionswechsel/Austritt).</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -977,6 +1569,63 @@
 3: Our plan is validated internally and actively communicated to all parties involved, ensuring good coordination between the players.
 4: We have a plan and we have already tested it.
 5: We regularly test and improve our plan, including the communication and coordination parts.</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>PRÉPARATION AUX INCIDENTS</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>INCIDENTVOORBEREIDING</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>VORFALLSBEREITSCHAFT</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Disposez-vous d'un plan de gestion des incidents ?</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Beschikt u over een incidentbeheerplan?</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>Haben Sie einen Vorfallsmanagementplan?</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>1 : Non, nous ne nous en sommes pas encore occupés.
+2 : Nous avons un plan, mais les responsabilités ne sont pas claires et nos fournisseurs n'ont pas été identifiés.
+3 : Notre plan est validé en interne et activement communiqué à toutes les parties impliquées, assurant une bonne coordination entre les acteurs.
+4 : Nous avons un plan et nous l'avons déjà testé.
+5 : Nous testons et améliorons régulièrement notre plan, y compris les aspects de communication et de coordination.</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>1: Nee, daar hebben we nog niet naar gekeken.
+2: We hebben een plan, maar de verantwoordelijkheden zijn niet duidelijk en onze leveranciers zijn niet geïdentificeerd.
+3: Ons plan is intern gevalideerd en actief gecommuniceerd aan alle betrokken partijen, wat zorgt voor een goede coördinatie tussen de spelers.
+4: We hebben een plan en we hebben het al getest.
+5: We testen en verbeteren regelmatig ons plan, inclusief de communicatie- en coördinatieonderdelen.</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>1: Nein, damit haben wir uns noch nicht befasst.
+2: Wir haben einen Plan, aber die Verantwortlichkeiten sind nicht klar und unsere Lieferanten wurden nicht identifiziert.
+3: Unser Plan ist intern validiert und wird aktiv an alle beteiligten Parteien kommuniziert, was eine gute Koordination zwischen den Akteuren gewährleistet.
+4: Wir haben einen Plan und haben ihn bereits getestet.
+5: Wir testen und verbessern regelmäßig unseren Plan, einschließlich der Kommunikations- und Koordinationsaspekte.</t>
         </is>
       </c>
     </row>
@@ -1029,7 +1678,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J6"/>
+  <dimension ref="A1:M6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1083,6 +1732,21 @@
           <t>description_doc[nl]</t>
         </is>
       </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>name[de]</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>description[de]</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>description_doc[de]</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="3" t="n">
@@ -1133,6 +1797,21 @@
           <t>Geen procesdocumentatie of niet formeel goedgekeurd door het management.</t>
         </is>
       </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Initial</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>Es gibt keinen Standardprozess.</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>Keine Prozessdokumentation oder nicht formell durch das Management genehmigt.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="n">
@@ -1183,6 +1862,21 @@
           <t>Er bestaat formeel goedgekeurde Procesdocumentatie, maar deze is de afgelopen 2 jaar niet herzien.</t>
         </is>
       </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Wiederholbar</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>Ein Ad-hoc-Prozess existiert und wird informell durchgeführt.</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>Es existiert eine formell genehmigte Prozessdokumentation, die jedoch in den letzten 2 Jahren nicht überprüft wurde.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="n">
@@ -1237,6 +1931,24 @@
       <c r="J4" s="3" t="inlineStr">
         <is>
           <t>Er bestaat formeel goedgekeurde procesdocumentatie en uitzonderingen worden gedocumenteerd en goedgekeurd. Gedocumenteerde en goedgekeurde uitzonderingen &lt; 5% van de tijd.</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Definiert</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>Ein formaler Prozess existiert und ist implementiert.
+Nachweise sind für die meisten Aktivitäten verfügbar.
+Weniger als 10% Prozessausnahmen.</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>Es existiert eine formell genehmigte Prozessdokumentation, und Ausnahmen sind dokumentiert und genehmigt.
+Dokumentierte und genehmigte Ausnahmen &lt; 5% der Fälle.</t>
         </is>
       </c>
     </row>
@@ -1300,6 +2012,26 @@
           <t>Er bestaat formeel goedgekeurde procesdocumentatie en uitzonderingen worden gedocumenteerd en goedgekeurd. Gedocumenteerde en goedgekeurde uitzonderingen &lt; 3% van de tijd.</t>
         </is>
       </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Gesteuert</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>Ein formaler Prozess existiert und ist implementiert.
+Nachweise sind für alle Aktivitäten verfügbar.
+Detaillierte Prozesskennzahlen werden erfasst und berichtet.
+Minimalziele für Kennzahlen wurden festgelegt.
+Weniger als 5% Prozessausnahmen.</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>Es existiert eine formell genehmigte Prozessdokumentation, und Ausnahmen sind dokumentiert und genehmigt.
+Dokumentierte und genehmigte Ausnahmen &lt; 3% der Fälle.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="n">
@@ -1361,6 +2093,26 @@
           <t>Er bestaat formeel goedgekeurde procesdocumentatie en uitzonderingen worden gedocumenteerd en goedgekeurd. Gedocumenteerde en goedgekeurde uitzonderingen &lt; 0,5% van de tijd.</t>
         </is>
       </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>Optimierend</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>Ein formaler Prozess existiert und ist implementiert.
+Nachweise sind für alle Aktivitäten verfügbar.
+Detaillierte Prozesskennzahlen werden erfasst und berichtet.
+Minimalziele für Kennzahlen wurden festgelegt und werden kontinuierlich verbessert.
+Weniger als 1% Prozessausnahmen.</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>Es existiert eine formell genehmigte Prozessdokumentation, und Ausnahmen sind dokumentiert und genehmigt.
+Dokumentierte und genehmigte Ausnahmen &lt; 0,5% der Fälle.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
feat(lib): add translations for cyfun-small-self-assessment (#3868)
</commit_message>
<xml_diff>
--- a/tools/excel/ccb/cyfun-small-self-assessment_new.xlsx
+++ b/tools/excel/ccb/cyfun-small-self-assessment_new.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="library_meta" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="requirements_meta" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="requirements_content" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="scores_meta" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="scores_content" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="library_meta" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="requirements_meta" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="requirements_content" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="scores_meta" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="scores_content" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -448,7 +448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:B17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -481,10 +481,8 @@
           <t>version</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="B3" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="4">
@@ -582,6 +580,84 @@
       <c r="B11" t="inlineStr">
         <is>
           <t>intuitem</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>name[fr]</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>CCB CyberFondamentaux Small - Auto-évaluation</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>name[nl]</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>CCB CyberFundamentals Small - Zelfbeoordeling</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>name[de]</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>CCB Cyber-Grundlagen Small - Selbstbewertung</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>description[fr]</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Centre pour la Cybersécurité Belgique - Cadre des CyberFondamentaux - Small
+Avec le contenu du site safeOnWeb en date de juillet 2025
+https://ccb.belgium.be</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>description[nl]</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Centrum voor Cyberveiligheid België - CyberFundamentals Framework - Small
+Met inhoud van de safeOnWeb website per juli 2025
+https://ccb.belgium.be</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>description[de]</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Zentrum für Cybersicherheit Belgien - Cyber-Grundlagen Framework - Small
+Mit Inhalten der safeOnWeb Website ab Juli 2025
+https://ccb.belgium.be</t>
         </is>
       </c>
     </row>
@@ -596,7 +672,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -704,6 +780,78 @@
       <c r="B9" t="inlineStr">
         <is>
           <t>scores</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>name[fr]</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>CCB CyberFondamentaux Small - Auto-évaluation</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>name[nl]</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>CCB CyberFundamentals Small - Zelfbeoordeling</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>name[de]</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>CCB Cyber-Grundlagen Small - Selbstbewertung</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>description[fr]</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Centre pour la Cybersécurité Belgique - Cadre des CyberFondamentaux - Small</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>description[nl]</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Centrum voor Cyberveiligheid België - CyberFundamentals Framework - Small</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>description[de]</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Zentrum für Cybersicherheit Belgien - Cyber-Grundlagen Framework - Small</t>
         </is>
       </c>
     </row>
@@ -718,7 +866,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:N9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -745,6 +893,51 @@
       <c r="E1" t="inlineStr">
         <is>
           <t>annotation</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>name[fr]</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>name[nl]</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>name[de]</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>description[fr]</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>description[nl]</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>description[de]</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>annotation[fr]</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>annotation[nl]</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>annotation[de]</t>
         </is>
       </c>
     </row>
@@ -776,6 +969,63 @@
 5: Two-factor authentication is in place for all critical systems.</t>
         </is>
       </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>MOTS DE PASSE</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>WACHTWOORDEN</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>PASSWÖRTER</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Avez-vous des règles en place pour vos mots de passe ?</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Heeft u regels voor uw wachtwoorden?</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Haben Sie Regeln für Ihre Passwörter?</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>1 : Pas de règles, les mots de passe n'ont aucun critère de création ou de réutilisation.
+2 : Il existe quelques règles concernant la création de mots de passe, mais pas de vérification de l'historique ou de la réutilisation.
+3 : Il existe des exigences communes pour tous les mots de passe et ceux-ci doivent être modifiés régulièrement.
+4 : Il existe des exigences strictes pour tous les utilisateurs et la plupart des systèmes, et les mots de passe ne sont modifiés qu'en cas d'indication de violation.
+5 : L'authentification multifactorielle est en place pour tous les systèmes critiques.</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>1: Geen regels, wachtwoorden hebben geen criteria voor aanmaak of hergebruik.
+2: Er zijn enkele regels rond het aanmaken van wachtwoorden, maar geen controle op geschiedenis of hergebruik.
+3: Er zijn gemeenschappelijke vereisten voor alle wachtwoorden en deze moeten regelmatig worden gewijzigd.
+4: Er zijn strenge vereisten voor alle gebruikers en de meeste systemen, en wachtwoorden worden alleen gewijzigd bij een indicatie van een schending.
+5: Multifactorauthenticatie is ingesteld voor alle kritieke systemen.</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>1: Keine Regeln, Passwörter haben keine Erstellungs- oder Wiederverwendungskriterien.
+2: Es gibt einige Regeln zur Passworterstellung, aber keine Überprüfung des Verlaufs oder der Wiederverwendung.
+3: Es gibt gemeinsame Anforderungen für alle Passwörter und diese sollten regelmäßig geändert werden.
+4: Es gibt strenge Anforderungen für alle Benutzer und die meisten Systeme, und Passwörter werden nur bei Anzeichen einer Verletzung geändert.
+5: Multi-Faktor-Authentifizierung ist für alle kritischen Systeme eingerichtet.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -805,6 +1055,63 @@
 5: All updates are done continuously and systematically, and are tested before implementation.</t>
         </is>
       </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>MAINTENANCE DES SYSTÈMES</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>SYSTEEMONDERHOUD</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>SYSTEMWARTUNG</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Mettez-vous à jour vos systèmes et applications ?</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Werkt u uw systemen en applicaties bij?</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Aktualisieren Sie Ihre Systeme und Anwendungen?</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>1 : Non, nous ne faisons aucune mise à jour tant que les systèmes continuent de fonctionner.
+2 : Des mises à jour manuelles sont effectuées en cas de besoin ou pour les systèmes les plus critiques.
+3 : Il existe une procédure standard pour la planification des mises à jour.
+4 : Tous les systèmes sont rapidement mis à jour vers leurs dernières versions.
+5 : Toutes les mises à jour sont effectuées de manière continue et systématique, et sont testées avant la mise en œuvre.</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>1: Nee, we doen geen updates zolang de systemen blijven werken.
+2: Handmatige updates worden gedaan wanneer dat nodig is of voor de meest kritieke systemen.
+3: Er is een standaardprocedure voor het plannen van updates.
+4: Alle systemen worden snel bijgewerkt naar de nieuwste versies.
+5: Alle updates worden continu en systematisch uitgevoerd en worden getest voor implementatie.</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>1: Nein, wir führen keine Updates durch, solange die Systeme weiter funktionieren.
+2: Manuelle Updates werden bei Bedarf oder für die kritischsten Systeme durchgeführt.
+3: Es gibt ein Standardverfahren für die Planung von Updates.
+4: Alle Systeme werden schnell auf die neuesten Versionen aktualisiert.
+5: Alle Updates werden kontinuierlich und systematisch durchgeführt und vor der Implementierung getestet.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -834,6 +1141,63 @@
 5: On all systems and updated daily. Suspicious activity is also reported.</t>
         </is>
       </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>GESTION ANTIVIRUS ET ANTI-MALWARE</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>ANTIVIRUS- EN ANTI-MALWAREBEHEER</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>ANTIVIRUS- UND ANTI-MALWARE-VERWALTUNG</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Disposez-vous d'un logiciel antivirus ou anti-malware ?</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Heeft u antivirus- of anti-malwaresoftware geïnstalleerd?</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Haben Sie Antivirus- oder Anti-Malware-Software installiert?</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>1 : Non, aucun.
+2 : Sur certains systèmes principaux, mais pas partout.
+3 : Sur tous les systèmes, mais ils ne sont pas nécessairement mis à jour.
+4 : Sur tous les systèmes et mis à jour plusieurs fois par semaine.
+5 : Sur tous les systèmes et mis à jour quotidiennement. Les activités suspectes sont également signalées.</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>1: Nee, geen.
+2: Op sommige belangrijke systemen, maar niet overal.
+3: Op alle systemen, maar ze worden niet noodzakelijk bijgewerkt.
+4: Op alle systemen en meerdere keren per week bijgewerkt.
+5: Op alle systemen en dagelijks bijgewerkt. Verdachte activiteiten worden ook gemeld.</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>1: Nein, keine.
+2: Auf einigen wichtigen Systemen, aber nicht überall.
+3: Auf allen Systemen, aber sie werden nicht unbedingt aktualisiert.
+4: Auf allen Systemen und mehrmals pro Woche aktualisiert.
+5: Auf allen Systemen und täglich aktualisiert. Verdächtige Aktivitäten werden ebenfalls gemeldet.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -863,6 +1227,63 @@
 5: The network is compartmentalized into strictly separated areas; anomalies are quickly detected and resolved.</t>
         </is>
       </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>SÉCURITÉ DU RÉSEAU</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>NETWERKBEVEILIGING</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>NETZWERKSICHERHEIT</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Protégez-vous votre réseau ?</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Beveiligt u uw netwerk?</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Schützen Sie Ihr Netzwerk?</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>1 : Pas activement : le réseau n'est pas segmenté et est connecté à internet sans mises à jour ni mots de passe forts.
+2 : De manière limitée : les réseaux public et interne sont séparés et protégés par un pare-feu.
+3 : Protection de base : un certain nombre de segmentations existent selon les fonctions et les besoins, et tout est documenté.
+4 : La sécurité du réseau est mesurée et surveillée ; les anomalies peuvent être détectées.
+5 : Le réseau est compartimenté en zones strictement séparées ; les anomalies sont rapidement détectées et résolues.</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>1: Niet actief: het netwerk is niet gesegmenteerd en is verbonden met het internet zonder updates en sterke wachtwoorden.
+2: Op een beperkte manier: het publieke en interne netwerk zijn gescheiden en beschermd door een firewall.
+3: Basisbescherming: er bestaan een aantal segmentaties volgens functies en behoeften en alles is gedocumenteerd.
+4: De beveiliging van het netwerk wordt gemeten en bewaakt; afwijkingen kunnen worden gedetecteerd.
+5: Het netwerk is opgedeeld in strikt gescheiden zones; afwijkingen worden snel gedetecteerd en opgelost.</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>1: Nicht aktiv: Das Netzwerk ist nicht segmentiert und ohne Updates und starke Passwörter mit dem Internet verbunden.
+2: In begrenztem Maße: Das öffentliche und das interne Netzwerk sind getrennt und durch eine Firewall geschützt.
+3: Grundschutz: Es gibt eine Reihe von Segmentierungen nach Funktionen und Bedürfnissen, und alles ist dokumentiert.
+4: Die Sicherheit des Netzwerks wird gemessen und überwacht; Anomalien können erkannt werden.
+5: Das Netzwerk ist in streng getrennte Bereiche unterteilt; Anomalien werden schnell erkannt und behoben.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -892,6 +1313,63 @@
 5: All data is backed up completely with fast recovery time and without data loss.</t>
         </is>
       </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>PROCÉDURE DE SAUVEGARDE</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>BACK-UPPROCEDURE</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>BACKUP-VERFAHREN</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Disposez-vous d'une procédure de sauvegarde ?</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Heeft u een back-upprocedure?</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>Haben Sie ein Backup-Verfahren?</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>1 : Non, ni systématique ni documentée.
+2 : Les sauvegardes sont limitées et manuelles, et la restauration n'est pas testée. Parfois, les sauvegardes sont faites localement par les employés eux-mêmes, sur des clés USB ou des disques durs externes.
+3 : Les sauvegardes sont testées et disponibles pour tous les systèmes principaux, et les restaurations de fichiers sont testées régulièrement.
+4 : Les sauvegardes sont chiffrées, disponibles pour tous les systèmes de l'organisation et testées immédiatement avec des indicateurs de performance à améliorer.
+5 : Toutes les données sont sauvegardées complètement avec un temps de récupération rapide et sans perte de données.</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>1: Nee, niet systematisch noch gedocumenteerd.
+2: Back-ups zijn beperkt en handmatig, en herstel wordt niet getest. Soms worden de back-ups lokaal door de medewerkers zelf gemaakt, op USB-sticks of externe harde schijven.
+3: Back-ups worden getest en zijn beschikbaar voor alle belangrijke systemen, en bestandsherstel wordt regelmatig getest.
+4: Back-ups zijn versleuteld, beschikbaar voor alle systemen in de organisatie en onmiddellijk getest met prestatie-indicatoren om te verbeteren.
+5: Alle gegevens worden volledig geback-upt met snelle hersteltijd en zonder gegevensverlies.</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>1: Nein, weder systematisch noch dokumentiert.
+2: Backups sind begrenzt und manuell, und die Wiederherstellung wird nicht getestet. Manchmal werden die Backups von den Mitarbeitern selbst lokal auf USB-Sticks oder externen Festplatten erstellt.
+3: Backups werden getestet und sind für alle wichtigen Systeme verfügbar, und Dateiwiederherstellungen werden regelmäßig getestet.
+4: Backups sind verschlüsselt, für alle Systeme in der Organisation verfügbar und werden sofort getestet, mit Leistungskennzahlen zur Verbesserung.
+5: Alle Daten werden vollständig gesichert mit schneller Wiederherstellungszeit und ohne Datenverlust.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -921,6 +1399,63 @@
 5: Administrator accounts are disabled or modified if there are changes and anomalies.</t>
         </is>
       </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>DROITS D'ADMINISTRATION</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>ADMINISTRATIERECHTEN</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>VERWALTUNGSRECHTE</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Comment protégez-vous vos comptes administrateur ?</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>Hoe beschermt u uw beheerdersaccounts?</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>Wie schützen Sie Ihre Administratorkonten?</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>1 : Sans vue d'ensemble de nos comptes administrateurs ; nous ne les protégeons pas spécifiquement.
+2 : Nous gérons l'accès administrateur uniquement sur certains services.
+3 : Tous les accès administrateur sont distribués dans des comptes séparés et gérés de manière centralisée.
+4 : Tous les comptes administrateur sont strictement surveillés avec des notifications automatiques en cas d'anomalies.
+5 : Les comptes administrateur sont désactivés ou modifiés en cas de changements et d'anomalies.</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>1: Zonder overzicht van onze beheerdersaccounts; we beschermen ze niet specifiek.
+2: We beheren beheerderstoegang alleen op bepaalde diensten.
+3: Alle beheerderstoegang is verdeeld over afzonderlijke accounts en wordt centraal beheerd.
+4: Alle beheerdersaccounts worden strikt bewaakt met automatische meldingen bij afwijkingen.
+5: Beheerdersaccounts worden uitgeschakeld of gewijzigd bij veranderingen en afwijkingen.</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>1: Ohne Überblick über unsere Administratorkonten; wir schützen sie nicht speziell.
+2: Wir verwalten den Administratorzugang nur bei bestimmten Diensten.
+3: Alle Administratorzugänge sind auf separate Konten verteilt und werden zentral verwaltet.
+4: Alle Administratorkonten werden streng überwacht, mit automatischen Benachrichtigungen bei Anomalien.
+5: Administratorkonten werden bei Änderungen und Anomalien deaktiviert oder geändert.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -950,6 +1485,63 @@
 5: Access control is centralized, regularly reviewed and follows the life cycle of employees (entry/change of position/exit).</t>
         </is>
       </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>SÉCURITÉ PHYSIQUE</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>FYSIEKE BEVEILIGING</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>PHYSISCHE SICHERHEIT</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Avez-vous des mesures en place pour protéger physiquement l'accès à vos locaux et à votre infrastructure ?</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Heeft u maatregelen getroffen om de fysieke toegang tot uw gebouwen en infrastructuur te beschermen?</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>Haben Sie Maßnahmen getroffen, um den physischen Zugang zu Ihren Räumlichkeiten und Ihrer Infrastruktur zu schützen?</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>1 : Nous n'avons rien en place.
+2 : Nous ne protégeons que les systèmes critiques (par ex. la salle des serveurs).
+3 : Toute notre infrastructure est protégée, y compris la protection contre les incendies et les inondations.
+4 : Nous contrôlons l'accès de manière centralisée (par ex. badges) et segmentons l'accès selon les niveaux de confidentialité.
+5 : Le contrôle d'accès est centralisé, régulièrement revu et suit le cycle de vie des employés (entrée/changement de poste/sortie).</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>1: We hebben niets in plaats.
+2: We beschermen alleen kritieke systemen (bijv. serverruimte).
+3: Al onze infrastructuur is beschermd, inclusief brand- en overstromingsbescherming.
+4: We controleren de toegang centraal (bijv. badges) en segmenteren de toegang op basis van vertrouwelijkheidsniveaus.
+5: Toegangscontrole is gecentraliseerd, wordt regelmatig herzien en volgt de levenscyclus van medewerkers (in dienst/functiewijziging/uit dienst).</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>1: Wir haben nichts eingerichtet.
+2: Wir schützen nur kritische Systeme (z.B. Serverraum).
+3: Unsere gesamte Infrastruktur ist geschützt, einschließlich Brand- und Hochwasserschutz.
+4: Wir kontrollieren den Zugang zentral (z.B. Badges) und segmentieren den Zugang nach Vertraulichkeitsstufen.
+5: Die Zugangskontrolle ist zentralisiert, wird regelmäßig überprüft und folgt dem Lebenszyklus der Mitarbeiter (Eintritt/Positionswechsel/Austritt).</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -977,6 +1569,63 @@
 3: Our plan is validated internally and actively communicated to all parties involved, ensuring good coordination between the players.
 4: We have a plan and we have already tested it.
 5: We regularly test and improve our plan, including the communication and coordination parts.</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>PRÉPARATION AUX INCIDENTS</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>INCIDENTVOORBEREIDING</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>VORFALLSBEREITSCHAFT</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Disposez-vous d'un plan de gestion des incidents ?</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Beschikt u over een incidentbeheerplan?</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>Haben Sie einen Vorfallsmanagementplan?</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>1 : Non, nous ne nous en sommes pas encore occupés.
+2 : Nous avons un plan, mais les responsabilités ne sont pas claires et nos fournisseurs n'ont pas été identifiés.
+3 : Notre plan est validé en interne et activement communiqué à toutes les parties impliquées, assurant une bonne coordination entre les acteurs.
+4 : Nous avons un plan et nous l'avons déjà testé.
+5 : Nous testons et améliorons régulièrement notre plan, y compris les aspects de communication et de coordination.</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>1: Nee, daar hebben we nog niet naar gekeken.
+2: We hebben een plan, maar de verantwoordelijkheden zijn niet duidelijk en onze leveranciers zijn niet geïdentificeerd.
+3: Ons plan is intern gevalideerd en actief gecommuniceerd aan alle betrokken partijen, wat zorgt voor een goede coördinatie tussen de spelers.
+4: We hebben een plan en we hebben het al getest.
+5: We testen en verbeteren regelmatig ons plan, inclusief de communicatie- en coördinatieonderdelen.</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>1: Nein, damit haben wir uns noch nicht befasst.
+2: Wir haben einen Plan, aber die Verantwortlichkeiten sind nicht klar und unsere Lieferanten wurden nicht identifiziert.
+3: Unser Plan ist intern validiert und wird aktiv an alle beteiligten Parteien kommuniziert, was eine gute Koordination zwischen den Akteuren gewährleistet.
+4: Wir haben einen Plan und haben ihn bereits getestet.
+5: Wir testen und verbessern regelmäßig unseren Plan, einschließlich der Kommunikations- und Koordinationsaspekte.</t>
         </is>
       </c>
     </row>
@@ -1029,7 +1678,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J6"/>
+  <dimension ref="A1:M6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1083,6 +1732,21 @@
           <t>description_doc[nl]</t>
         </is>
       </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>name[de]</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>description[de]</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>description_doc[de]</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="3" t="n">
@@ -1133,6 +1797,21 @@
           <t>Geen procesdocumentatie of niet formeel goedgekeurd door het management.</t>
         </is>
       </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Initial</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>Es gibt keinen Standardprozess.</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>Keine Prozessdokumentation oder nicht formell durch das Management genehmigt.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="n">
@@ -1183,6 +1862,21 @@
           <t>Er bestaat formeel goedgekeurde Procesdocumentatie, maar deze is de afgelopen 2 jaar niet herzien.</t>
         </is>
       </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Wiederholbar</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>Ein Ad-hoc-Prozess existiert und wird informell durchgeführt.</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>Es existiert eine formell genehmigte Prozessdokumentation, die jedoch in den letzten 2 Jahren nicht überprüft wurde.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="n">
@@ -1237,6 +1931,24 @@
       <c r="J4" s="3" t="inlineStr">
         <is>
           <t>Er bestaat formeel goedgekeurde procesdocumentatie en uitzonderingen worden gedocumenteerd en goedgekeurd. Gedocumenteerde en goedgekeurde uitzonderingen &lt; 5% van de tijd.</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Definiert</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>Ein formaler Prozess existiert und ist implementiert.
+Nachweise sind für die meisten Aktivitäten verfügbar.
+Weniger als 10% Prozessausnahmen.</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>Es existiert eine formell genehmigte Prozessdokumentation, und Ausnahmen sind dokumentiert und genehmigt.
+Dokumentierte und genehmigte Ausnahmen &lt; 5% der Fälle.</t>
         </is>
       </c>
     </row>
@@ -1300,6 +2012,26 @@
           <t>Er bestaat formeel goedgekeurde procesdocumentatie en uitzonderingen worden gedocumenteerd en goedgekeurd. Gedocumenteerde en goedgekeurde uitzonderingen &lt; 3% van de tijd.</t>
         </is>
       </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Gesteuert</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>Ein formaler Prozess existiert und ist implementiert.
+Nachweise sind für alle Aktivitäten verfügbar.
+Detaillierte Prozesskennzahlen werden erfasst und berichtet.
+Minimalziele für Kennzahlen wurden festgelegt.
+Weniger als 5% Prozessausnahmen.</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>Es existiert eine formell genehmigte Prozessdokumentation, und Ausnahmen sind dokumentiert und genehmigt.
+Dokumentierte und genehmigte Ausnahmen &lt; 3% der Fälle.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="n">
@@ -1361,6 +2093,26 @@
           <t>Er bestaat formeel goedgekeurde procesdocumentatie en uitzonderingen worden gedocumenteerd en goedgekeurd. Gedocumenteerde en goedgekeurde uitzonderingen &lt; 0,5% van de tijd.</t>
         </is>
       </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>Optimierend</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>Ein formaler Prozess existiert und ist implementiert.
+Nachweise sind für alle Aktivitäten verfügbar.
+Detaillierte Prozesskennzahlen werden erfasst und berichtet.
+Minimalziele für Kennzahlen wurden festgelegt und werden kontinuierlich verbessert.
+Weniger als 1% Prozessausnahmen.</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>Es existiert eine formell genehmigte Prozessdokumentation, und Ausnahmen sind dokumentiert und genehmigt.
+Dokumentierte und genehmigte Ausnahmen &lt; 0,5% der Fälle.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>